<commit_message>
Prep report update and capping individually
</commit_message>
<xml_diff>
--- a/data/country_baselines/Updated/Copy of Baseline_information_template_Eswatini_ 09 Jul 2026.xlsx
+++ b/data/country_baselines/Updated/Copy of Baseline_information_template_Eswatini_ 09 Jul 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Setsabile Gulwako\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/country_baselines/Updated/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7172823F-9488-4D7B-AEE9-C9E1D8366F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{7172823F-9488-4D7B-AEE9-C9E1D8366F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFCACFD8-7998-C248-9C88-F88607FB2095}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -181,7 +181,7 @@
     <numFmt numFmtId="164" formatCode="0.0&quot;%&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -210,12 +210,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -354,6 +348,8 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -365,12 +361,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -717,14 +711,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G38"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="68.25" customWidth="1"/>
+    <col min="1" max="1" width="68.1640625" customWidth="1"/>
     <col min="2" max="2" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.58203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -735,14 +729,14 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -752,13 +746,13 @@
       <c r="C3" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="9"/>
-      <c r="G3" s="10"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="F3" s="11"/>
+      <c r="G3" s="12"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -768,11 +762,11 @@
       <c r="C4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="11"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="13"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="E4" s="13"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="15"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -782,11 +776,11 @@
       <c r="C5" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="13"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="E5" s="13"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="15"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -796,11 +790,11 @@
       <c r="C6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="11"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="13"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="E6" s="13"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="15"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -810,11 +804,11 @@
       <c r="C7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="13"/>
-    </row>
-    <row r="8" spans="1:7" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="E7" s="13"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="15"/>
+    </row>
+    <row r="8" spans="1:7" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
@@ -824,11 +818,11 @@
       <c r="C8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="14"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="16"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="E8" s="16"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="18"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -839,35 +833,35 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>33</v>
       </c>
@@ -878,177 +872,180 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="1"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B17" s="3"/>
     </row>
-    <row r="18" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="9">
         <v>0.222</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="18">
+      <c r="B20" s="9">
         <v>0.49399999999999999</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="9">
         <v>0.28399999999999997</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="18">
+      <c r="B22" s="9">
         <v>0</v>
       </c>
       <c r="C22" s="1"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="18">
+      <c r="B23" s="9">
         <v>2.3E-2</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B24" s="4"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="18">
+      <c r="B25" s="9">
         <v>0.92200000000000004</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="18">
+      <c r="B26" s="9">
         <v>0.64200000000000002</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="18">
+      <c r="B27" s="9">
         <v>0.36199999999999999</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="29" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D27" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="1"/>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="1"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B31" s="3"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="1"/>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B33" s="17">
+      <c r="B33" s="8">
         <v>0.95</v>
       </c>
       <c r="C33" s="1"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="17"/>
+      <c r="B34" s="8"/>
       <c r="C34" s="1"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="17"/>
+      <c r="B35" s="8"/>
       <c r="C35" s="1"/>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="17">
+      <c r="B36" s="8">
         <v>0.96</v>
       </c>
       <c r="C36" s="1"/>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B37" s="17"/>
+      <c r="B37" s="8"/>
       <c r="C37" s="1"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B38" s="4"/>
     </row>
   </sheetData>

</xml_diff>